<commit_message>
atualização do codigo da forquilha
</commit_message>
<xml_diff>
--- a/dados-catalago-pcm-externo/nomes_usuais.xlsx
+++ b/dados-catalago-pcm-externo/nomes_usuais.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amaggicombr-my.sharepoint.com/personal/hiago_andre_amaggi_com_br/Documents/Área de Trabalho/codigos/catalogoPecas/dados-catalago-pcm-externo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="108" documentId="11_AD4D361C20488DEA4E38A03414D973025ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28A4B06B-14B7-492E-AA3C-165EBFCAD48F}"/>
+  <xr:revisionPtr revIDLastSave="112" documentId="11_AD4D361C20488DEA4E38A03414D973025ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37358B64-4CD0-47DB-B59C-9FF9808AADAA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1363,7 +1363,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2853,8 +2855,8 @@
       </c>
     </row>
     <row r="110" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A110" s="5">
-        <v>64262</v>
+      <c r="A110" s="18">
+        <v>1010051726</v>
       </c>
       <c r="B110" s="5" t="s">
         <v>112</v>
@@ -2885,7 +2887,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" s="5">
         <v>1040077370</v>
       </c>
@@ -2895,8 +2897,9 @@
       <c r="C113" s="6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G113" s="15"/>
+    </row>
+    <row r="114" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" s="5">
         <v>1040099247</v>
       </c>
@@ -2907,7 +2910,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" s="5">
         <v>1040100560</v>
       </c>
@@ -2918,7 +2921,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A116" s="5">
         <v>1040077399</v>
       </c>
@@ -2929,7 +2932,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A117" s="5">
         <v>1040077374</v>
       </c>
@@ -2940,7 +2943,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A118" s="5">
         <v>1040077399</v>
       </c>
@@ -2951,7 +2954,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" s="16">
         <v>1010050632</v>
       </c>
@@ -2962,7 +2965,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="120" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A120" s="5">
         <v>409250</v>
       </c>
@@ -2973,7 +2976,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A121" s="5">
         <v>1010020541</v>
       </c>
@@ -2984,7 +2987,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A122" s="5">
         <v>1010020879</v>
       </c>
@@ -2995,7 +2998,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A123" s="5">
         <v>1040077380</v>
       </c>
@@ -3006,7 +3009,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A124" s="5">
         <v>1010021520</v>
       </c>
@@ -3017,7 +3020,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A125" s="5">
         <v>1040098861</v>
       </c>
@@ -3028,7 +3031,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A126" s="5">
         <v>1010077261</v>
       </c>
@@ -3039,7 +3042,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A127" s="5">
         <v>1010027664</v>
       </c>
@@ -3050,7 +3053,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A128" s="5">
         <v>1010083731</v>
       </c>
@@ -5052,7 +5055,6 @@
       <c r="C309" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="F309" s="18"/>
     </row>
     <row r="310" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A310" s="12">

</xml_diff>